<commit_message>
Fixed a typo in one of the raw data files.
</commit_message>
<xml_diff>
--- a/formatted_raw/2-24-25_ZS_R4100&R16_LN.xlsx
+++ b/formatted_raw/2-24-25_ZS_R4100&R16_LN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rowde002\Desktop\Graphs With Gage Version 4\formatted_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D293E8E-A1D4-43AA-8FD2-69B0568FC31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A7538E-D622-4F01-86BF-B75030E22184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6495" yWindow="2010" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Microplate Cycle 1 (0 h)" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="272">
   <si>
     <t>Sample IDs</t>
   </si>
@@ -845,15 +845,6 @@
     <t>NQ-R4100-LN-1000</t>
   </si>
   <si>
-    <t>NQ-R4100-LN-1001</t>
-  </si>
-  <si>
-    <t>NQ-R4100-LN-1002</t>
-  </si>
-  <si>
-    <t>NQ-R4100-LN-1003</t>
-  </si>
-  <si>
     <t>RT-R16-LN-100000</t>
   </si>
 </sst>
@@ -1381,7 +1372,18 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
-    <col min="2" max="14" width="8.5703125" customWidth="1"/>
+    <col min="2" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
     <col min="15" max="15" width="33.7109375" customWidth="1"/>
     <col min="16" max="26" width="8.5703125" customWidth="1"/>
   </cols>
@@ -1511,7 +1513,7 @@
         <v>12</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="O16" s="11" t="s">
         <v>40</v>
@@ -1555,7 +1557,7 @@
         <v>12</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="O17" s="7" t="s">
         <v>41</v>
@@ -1599,7 +1601,7 @@
         <v>12</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="O18" s="11" t="s">
         <v>42</v>
@@ -1643,7 +1645,7 @@
         <v>12</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="O19" s="11" t="s">
         <v>43</v>
@@ -1708,7 +1710,7 @@
         <v>20</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>21</v>
@@ -1749,7 +1751,7 @@
         <v>20</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>21</v>
@@ -1790,7 +1792,7 @@
         <v>20</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>21</v>

</xml_diff>